<commit_message>
feat(corporate-legal-english): add consolidated dealroom PDF
</commit_message>
<xml_diff>
--- a/testakten/gesellschaftsrecht-legal-english-frankfurt-startup/18-cap-table-und-waterfall.xlsx
+++ b/testakten/gesellschaftsrecht-legal-english-frankfurt-startup/18-cap-table-und-waterfall.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waterfall" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
 </file>
 
@@ -100,7 +100,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -130,6 +130,21 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -553,7 +568,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>21.05.2026</t>
+          <t>28.05.2026</t>
         </is>
       </c>
     </row>
@@ -565,7 +580,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Dieses Arbeitsmodell zeigt den Cap Table der Kometenfalter Systems GmbH vor und nach Closing der Series A, die Pool-Szenarien pre- und post-money, das Wandeldarlehen von Frau Ermelind und den Exit-Waterfall der Series A Liquidation Preference.</t>
+          <t>Dieses Arbeitsmodell zeigt den Cap Table der Kometenfalter Systems GmbH vor und nach Closing der Series A, die Pool-Szenarien pre- und post-money, das Wandeldarlehen der Tante Ermelind Capital UG und den Exit-Waterfall der Series-A-Liquidation-Preference.</t>
         </is>
       </c>
     </row>
@@ -577,7 +592,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Die Zahlen sind Arbeitsannahmen der Kanzlei auf Basis des Term Sheet vom 19.05.2026 und des Cap-Table-Excels der Mandantin. Vor Eingang der endgültigen Kapitalerhöhungsbeschlüsse, der angepassten Gesellschafterliste und des Notar-Termins sind sämtliche Werte vorläufig.</t>
+          <t>Die Zahlen sind Arbeitsannahmen der Kanzlei auf Basis des Term Sheet vom 14.05.2026, des Cap Table v19 und der offenen CFO-Abstimmung vom 28.05.2026. Vor Eingang der endgültigen Kapitalerhöhungsbeschlüsse, der angepassten Gesellschafterliste und des Notar-Termins sind sämtliche Werte vorläufig.</t>
         </is>
       </c>
     </row>
@@ -589,7 +604,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Term Sheet (Datei 03), SHA/Satzung/Vesting (Datei 04), Wandeldarlehen Frau Ermelind (Datei 10), Closing-Checkliste (Datei 15).</t>
+          <t>Term Sheet (Datei 03), Cap Table/Gesellschafterliste (Datei 02), Wandeldarlehen Tante Ermelind (Datei 10), Closing-Checkliste (Datei 15).</t>
         </is>
       </c>
     </row>
@@ -607,7 +622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -617,7 +632,7 @@
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="52" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -670,314 +685,351 @@
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>Gründerin Wendelgard</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Kunigunde Reiter</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>Gesellschafterliste</t>
         </is>
       </c>
-      <c r="C4" s="5" t="n">
+      <c r="C4" s="17" t="n">
         <v>12000</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="D4" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="17">
         <f>C4+D4</f>
         <v/>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="13">
         <f>E4/SUM($E$4:$E$10)</f>
         <v/>
       </c>
-      <c r="G4" s="6">
-        <f>E4/SUM($E$4:$E$11)</f>
+      <c r="G4" s="13">
+        <f>E4/SUM($E$4:$E$12)</f>
         <v/>
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>formell und wirtschaftlich relevant</t>
+          <t>Gründerin CEO, formell und wirtschaftlich relevant</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Gründer Kunibert</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Meinhard Voss</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>Gesellschafterliste</t>
         </is>
       </c>
-      <c r="C5" s="5" t="n">
+      <c r="C5" s="17" t="n">
         <v>9000</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="D5" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="17">
         <f>C5+D5</f>
         <v/>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="13">
         <f>E5/SUM($E$4:$E$10)</f>
         <v/>
       </c>
-      <c r="G5" s="6">
-        <f>E5/SUM($E$4:$E$11)</f>
+      <c r="G5" s="13">
+        <f>E5/SUM($E$4:$E$12)</f>
         <v/>
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>formell und wirtschaftlich relevant</t>
+          <t>Gründer CTO, formell und wirtschaftlich relevant</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Walburga Stein</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Gesellschafterliste</t>
+        </is>
+      </c>
+      <c r="C6" s="17" t="n">
+        <v>6000</v>
+      </c>
+      <c r="D6" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="17">
+        <f>C6+D6</f>
+        <v/>
+      </c>
+      <c r="F6" s="13">
+        <f>E6/SUM($E$4:$E$10)</f>
+        <v/>
+      </c>
+      <c r="G6" s="13">
+        <f>E6/SUM($E$4:$E$12)</f>
+        <v/>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>Gründerin Product, formell und wirtschaftlich relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Stahlauge Ventures GmbH</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Gesellschafterliste</t>
         </is>
       </c>
-      <c r="C6" s="5" t="n">
-        <v>6000</v>
-      </c>
-      <c r="D6" s="5" t="n">
+      <c r="C7" s="17" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D7" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="5">
-        <f>C6+D6</f>
-        <v/>
-      </c>
-      <c r="F6" s="6">
-        <f>E6/SUM($E$4:$E$10)</f>
-        <v/>
-      </c>
-      <c r="G6" s="6">
-        <f>E6/SUM($E$4:$E$11)</f>
-        <v/>
-      </c>
-      <c r="H6" s="7" t="inlineStr">
-        <is>
-          <t>Seed-Rechte (Information Rights, Tag-along) prüfen</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Krämer Angel Pool GbR</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Gesellschafterliste</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="n">
-        <v>3000</v>
-      </c>
-      <c r="D7" s="5" t="n">
+      <c r="E7" s="17">
+        <f>C7+D7</f>
+        <v/>
+      </c>
+      <c r="F7" s="13">
+        <f>E7/SUM($E$4:$E$10)</f>
+        <v/>
+      </c>
+      <c r="G7" s="13">
+        <f>E7/SUM($E$4:$E$12)</f>
+        <v/>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Seed-Investor; 1x non-participating preference im Seed-SHA behauptet</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Bestehender VSOP</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>nur Cap Table</t>
+        </is>
+      </c>
+      <c r="C8" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="5">
-        <f>C7+D7</f>
-        <v/>
-      </c>
-      <c r="F7" s="6">
-        <f>E7/SUM($E$4:$E$10)</f>
-        <v/>
-      </c>
-      <c r="G7" s="6">
-        <f>E7/SUM($E$4:$E$11)</f>
-        <v/>
-      </c>
-      <c r="H7" s="7" t="inlineStr">
-        <is>
-          <t>GbR-Vertretung und Zustimmung der Gesellschafter prüfen</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Bestehender VSOP</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="D8" s="17" t="n">
+        <v>900</v>
+      </c>
+      <c r="E8" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>separat</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>separat</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>virtuell, 900 zugesagt, davon 360 vested; separater Informationsblock, in V19b nicht in der FD-Summe</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Option Pool reserviert</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>nur Cap Table</t>
         </is>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C9" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="D8" s="5" t="n">
-        <v>2400</v>
-      </c>
-      <c r="E8" s="5">
-        <f>C8+D8</f>
-        <v/>
-      </c>
-      <c r="F8" s="6">
-        <f>E8/SUM($E$4:$E$10)</f>
-        <v/>
-      </c>
-      <c r="G8" s="6">
-        <f>E8/SUM($E$4:$E$11)</f>
-        <v/>
-      </c>
-      <c r="H8" s="7" t="inlineStr">
-        <is>
-          <t>virtuell, aber Exit-relevant</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Pool-Erhöhung Series A</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="D9" s="17" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E9" s="17">
+        <f>C9+D9</f>
+        <v/>
+      </c>
+      <c r="F9" s="13">
+        <f>E9/SUM($E$4:$E$10)</f>
+        <v/>
+      </c>
+      <c r="G9" s="13">
+        <f>E9/SUM($E$4:$E$12)</f>
+        <v/>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Pool-Shuffle: 12 Prozent fully diluted pre-money, hier auf 5.000 gerundet</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Tante Ermelind aus Wandlung</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>nur Cap Table</t>
         </is>
       </c>
-      <c r="C9" s="5" t="n">
+      <c r="C10" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="D9" s="5" t="n">
-        <v>3000</v>
-      </c>
-      <c r="E9" s="5">
-        <f>C9+D9</f>
-        <v/>
-      </c>
-      <c r="F9" s="6">
-        <f>E9/SUM($E$4:$E$10)</f>
-        <v/>
-      </c>
-      <c r="G9" s="6">
-        <f>E9/SUM($E$4:$E$11)</f>
-        <v/>
-      </c>
-      <c r="H9" s="7" t="inlineStr">
-        <is>
-          <t>Pool Shuffle: Lastenverteilung Altgesellschafter / Investoren</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>Wandeldarlehen Frau Ermelind</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>nur Cap Table</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="n">
+      <c r="D10" s="17" t="n">
+        <v>6700</v>
+      </c>
+      <c r="E10" s="17">
+        <f>C10+D10</f>
+        <v/>
+      </c>
+      <c r="F10" s="13">
+        <f>E10/SUM($E$4:$E$10)</f>
+        <v/>
+      </c>
+      <c r="G10" s="13">
+        <f>E10/SUM($E$4:$E$12)</f>
+        <v/>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Convertible; Cap greift gegenüber Discount, Arbeitswert laut Datei 02</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Series A Northbridge</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Kapitalerhöhung bei Closing</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="5" t="n">
-        <v>1750</v>
-      </c>
-      <c r="E10" s="5">
-        <f>C10+D10</f>
-        <v/>
-      </c>
-      <c r="F10" s="6">
-        <f>E10/SUM($E$4:$E$10)</f>
-        <v/>
-      </c>
-      <c r="G10" s="6">
-        <f>E10/SUM($E$4:$E$11)</f>
-        <v/>
-      </c>
-      <c r="H10" s="7" t="inlineStr">
-        <is>
-          <t>Discount/Cap-Szenario gemäß Wandeldarlehensvertrag vom 14.08.2024</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Series A Investoren</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="D11" s="17" t="n">
+        <v>16679</v>
+      </c>
+      <c r="E11" s="17">
+        <f>C11+D11</f>
+        <v/>
+      </c>
+      <c r="F11" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G11" s="13">
+        <f>E11/SUM($E$4:$E$12)</f>
+        <v/>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Lead Investor; 4,8 Mio. EUR von 5,2 Mio. EUR Subscription</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Series A Krämer Angels</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Kapitalerhöhung bei Closing</t>
         </is>
       </c>
-      <c r="C11" s="5" t="n">
+      <c r="C12" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="D11" s="5" t="n">
-        <v>13000</v>
-      </c>
-      <c r="E11" s="5">
-        <f>C11+D11</f>
-        <v/>
-      </c>
-      <c r="F11" s="8" t="inlineStr">
+      <c r="D12" s="17" t="n">
+        <v>1390</v>
+      </c>
+      <c r="E12" s="17">
+        <f>C12+D12</f>
+        <v/>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G11" s="6">
-        <f>E11/SUM($E$4:$E$11)</f>
-        <v/>
-      </c>
-      <c r="H11" s="7" t="inlineStr">
-        <is>
-          <t>erst nach notarieller Kapitalerhöhung und Eintragung im Handelsregister</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="G12" s="13">
+        <f>E12/SUM($E$4:$E$12)</f>
+        <v/>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Co-Investor-Pool; 0,4 Mio. EUR Subscription</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>Summe</t>
         </is>
       </c>
-      <c r="B12" s="10" t="n"/>
-      <c r="C12" s="9">
-        <f>SUM(C4:C11)</f>
-        <v/>
-      </c>
-      <c r="D12" s="9">
-        <f>SUM(D4:D11)</f>
-        <v/>
-      </c>
-      <c r="E12" s="9">
-        <f>SUM(E4:E11)</f>
-        <v/>
-      </c>
-      <c r="F12" s="11">
-        <f>SUM(F4:F10)</f>
-        <v/>
-      </c>
-      <c r="G12" s="11">
-        <f>SUM(G4:G11)</f>
-        <v/>
-      </c>
-      <c r="H12" s="10" t="n"/>
+      <c r="B13" s="7" t="n"/>
+      <c r="C13" s="17">
+        <f>SUM(C4:C12)</f>
+        <v/>
+      </c>
+      <c r="D13" s="17">
+        <f>SUM(D4:D12)</f>
+        <v/>
+      </c>
+      <c r="E13" s="17">
+        <f>SUM(E4:E12)</f>
+        <v/>
+      </c>
+      <c r="F13" s="13">
+        <f>SUM(F4:F7,F9:F10)</f>
+        <v/>
+      </c>
+      <c r="G13" s="13">
+        <f>SUM(G4:G7,G9:G12)</f>
+        <v/>
+      </c>
+      <c r="H13" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1043,8 +1095,9 @@
           <t>A: Pool pre-money</t>
         </is>
       </c>
-      <c r="B4" s="13" t="n">
-        <v>0.3023</v>
+      <c r="B4" s="13">
+        <f>SUM('Cap Table'!E11:E12)/'Cap Table'!E13</f>
+        <v/>
       </c>
       <c r="C4" s="13" t="n">
         <v>0.12</v>
@@ -1066,8 +1119,9 @@
           <t>B: Pool post-money</t>
         </is>
       </c>
-      <c r="B5" s="13" t="n">
-        <v>0.3023</v>
+      <c r="B5" s="13">
+        <f>SUM('Cap Table'!E11:E12)/'Cap Table'!E13</f>
+        <v/>
       </c>
       <c r="C5" s="13" t="n">
         <v>0.12</v>
@@ -1079,7 +1133,7 @@
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>Investor wird am Pool-Aufbau beteiligt; Position der Investoren wirtschaftlich nachteiliger.</t>
+          <t>Investor wird am Pool-Aufbau beteiligt; Gründerposition wirtschaftlich etwas weniger belastet.</t>
         </is>
       </c>
     </row>
@@ -1097,7 +1151,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1111,7 +1165,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Wandeldarlehen Frau Ermelind: Discount vs. Valuation Cap</t>
+          <t>Wandeldarlehen Tante Ermelind: Discount vs. Valuation Cap</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1253,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>1.25</v>
+        <v>1.5</v>
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
@@ -1213,7 +1267,7 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>vor Term-Sheet-Annahme Zahlenprobe machen</t>
+          <t>Arbeitswert; genaue Zinstage vor Closing mit Zahlungsdatum abstimmen</t>
         </is>
       </c>
     </row>
@@ -1266,6 +1320,32 @@
       </c>
       <c r="B11" s="15" t="n">
         <v>5200000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>Arbeitswert Cap Table</t>
+        </is>
+      </c>
+      <c r="B12" s="20" t="n">
+        <v>6700</v>
+      </c>
+      <c r="C12" s="21" t="n"/>
+      <c r="D12" s="21" t="inlineStr">
+        <is>
+          <t>Aus Datei 02</t>
+        </is>
+      </c>
+      <c r="E12" s="21" t="inlineStr">
+        <is>
+          <t>gerundete Wandlungsanteile im V19b-Szenario</t>
+        </is>
+      </c>
+      <c r="F12" s="21" t="inlineStr">
+        <is>
+          <t>Senior-Review vor Außenkommunikation</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1343,8 +1423,9 @@
         <f>B4</f>
         <v/>
       </c>
-      <c r="D4" s="6" t="n">
-        <v>0.3023</v>
+      <c r="D4" s="6">
+        <f>SUM('Cap Table'!E11:E12)/'Cap Table'!E13</f>
+        <v/>
       </c>
       <c r="E4" s="15">
         <f>MAX(C4,A4*D4)</f>
@@ -1366,8 +1447,9 @@
         <f>B5</f>
         <v/>
       </c>
-      <c r="D5" s="6" t="n">
-        <v>0.3023</v>
+      <c r="D5" s="6">
+        <f>SUM('Cap Table'!E11:E12)/'Cap Table'!E13</f>
+        <v/>
       </c>
       <c r="E5" s="15">
         <f>MAX(C5,A5*D5)</f>
@@ -1389,8 +1471,9 @@
         <f>B6</f>
         <v/>
       </c>
-      <c r="D6" s="6" t="n">
-        <v>0.3023</v>
+      <c r="D6" s="6">
+        <f>SUM('Cap Table'!E11:E12)/'Cap Table'!E13</f>
+        <v/>
       </c>
       <c r="E6" s="15">
         <f>MAX(C6,A6*D6)</f>
@@ -1412,8 +1495,9 @@
         <f>B7</f>
         <v/>
       </c>
-      <c r="D7" s="6" t="n">
-        <v>0.3023</v>
+      <c r="D7" s="6">
+        <f>SUM('Cap Table'!E11:E12)/'Cap Table'!E13</f>
+        <v/>
       </c>
       <c r="E7" s="15">
         <f>MAX(C7,A7*D7)</f>
@@ -1435,8 +1519,9 @@
         <f>B8</f>
         <v/>
       </c>
-      <c r="D8" s="6" t="n">
-        <v>0.3023</v>
+      <c r="D8" s="6">
+        <f>SUM('Cap Table'!E11:E12)/'Cap Table'!E13</f>
+        <v/>
       </c>
       <c r="E8" s="15">
         <f>MAX(C8,A8*D8)</f>

</xml_diff>